<commit_message>
Marcar atividade 503 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2197,13 +2197,17 @@
         <v>40</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-09-13 01:19</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">

</xml_diff>

<commit_message>
Marcar atividade 500 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2059,13 +2059,17 @@
         <v>20</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-09-13 01:19</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">

</xml_diff>

<commit_message>
Marcar atividade 501 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2109,13 +2109,17 @@
         <v>30</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-09-13 01:21</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">

</xml_diff>

<commit_message>
Marcar atividade 491 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -1617,13 +1617,17 @@
         <v>20</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-09-13 18:16</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">

</xml_diff>

<commit_message>
Marcar atividade 506 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2351,13 +2351,17 @@
         <v>30</v>
       </c>
       <c r="I39" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-09-14 03:44</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">

</xml_diff>

<commit_message>
Marcar atividade 509 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2493,13 +2493,17 @@
         <v>30</v>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-09-14 10:41</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">

</xml_diff>

<commit_message>
Marcar atividade 505 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2305,13 +2305,17 @@
         <v>10</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-09-14 10:55</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">

</xml_diff>

<commit_message>
Marcar atividade 508 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2451,13 +2451,17 @@
         <v>20</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-09-14 22:38</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">

</xml_diff>

<commit_message>
Marcar atividade 511 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2597,13 +2597,17 @@
         <v>40</v>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-09-15 00:40</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">

</xml_diff>

<commit_message>
Marcar atividade 498 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -1967,13 +1967,17 @@
         <v>20</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-09-15 01:34</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">

</xml_diff>

<commit_message>
Marcar atividade 504 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2263,13 +2263,17 @@
         <v>30</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-09-15 03:06</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">

</xml_diff>

<commit_message>
Marcar atividade 513 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2701,13 +2701,17 @@
         <v>20</v>
       </c>
       <c r="I46" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J46" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>2026-09-15 11:59</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">

</xml_diff>

<commit_message>
Marcar atividade 502 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2167,13 +2167,17 @@
         <v>20</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-09-16 03:20</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">

</xml_diff>

<commit_message>
Marcar atividade 514 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2755,13 +2755,17 @@
         <v>30</v>
       </c>
       <c r="I47" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J47" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-09-16 10:58</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">

</xml_diff>

<commit_message>
Marcar atividade 512 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2659,13 +2659,17 @@
         <v>40</v>
       </c>
       <c r="I45" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J45" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>2026-09-17 02:43</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">

</xml_diff>

<commit_message>
Marcar atividade 497 como pendente
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -1920,14 +1920,10 @@
         <v>30</v>
       </c>
       <c r="J30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>2026-09-11 16:14</t>
-        </is>
-      </c>
+      <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">

</xml_diff>

<commit_message>
Marcar atividade 498 como pendente
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -1966,14 +1966,10 @@
         <v>20</v>
       </c>
       <c r="J31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>2026-09-15 01:34</t>
-        </is>
-      </c>
+      <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">

</xml_diff>

<commit_message>
Marcar atividade 499 como pendente
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2012,14 +2012,10 @@
         <v>45</v>
       </c>
       <c r="J32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>2026-09-11 18:44</t>
-        </is>
-      </c>
+      <c r="L32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">

</xml_diff>

<commit_message>
Marcar atividade 500 como pendente
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2058,14 +2058,10 @@
         <v>20</v>
       </c>
       <c r="J33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>2026-09-13 01:19</t>
-        </is>
-      </c>
+      <c r="L33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">

</xml_diff>

<commit_message>
Marcar atividade 499 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -1920,10 +1920,14 @@
         <v>30</v>
       </c>
       <c r="J30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-09-17 12:45</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1966,10 +1970,14 @@
         <v>20</v>
       </c>
       <c r="J31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-09-17 12:45</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2012,10 +2020,14 @@
         <v>45</v>
       </c>
       <c r="J32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-09-17 12:45</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">

</xml_diff>

<commit_message>
Marcar atividade 507 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2417,13 +2417,17 @@
         <v>20</v>
       </c>
       <c r="I40" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-09-17 16:46</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">

</xml_diff>

<commit_message>
Marcar atividade 515 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2813,13 +2813,17 @@
         <v>20</v>
       </c>
       <c r="I48" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J48" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-09-18 04:13</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">

</xml_diff>

<commit_message>
Adicionar atividade: English Life - Conversação em grupo (Darlei Delfino)
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1937"/>
+  <dimension ref="A1:L1938"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -89778,6 +89778,52 @@
       </c>
       <c r="K1937" t="inlineStr"/>
       <c r="L1937" t="inlineStr"/>
+    </row>
+    <row r="1938">
+      <c r="A1938" t="n">
+        <v>3862</v>
+      </c>
+      <c r="B1938" t="inlineStr">
+        <is>
+          <t>Darlei Delfino</t>
+        </is>
+      </c>
+      <c r="C1938" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="D1938" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="E1938" t="inlineStr">
+        <is>
+          <t>English Life - Conversação em grupo</t>
+        </is>
+      </c>
+      <c r="F1938" t="inlineStr">
+        <is>
+          <t>Speaking</t>
+        </is>
+      </c>
+      <c r="G1938" t="inlineStr">
+        <is>
+          <t>English Live</t>
+        </is>
+      </c>
+      <c r="H1938" t="n">
+        <v>45</v>
+      </c>
+      <c r="I1938" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1938" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1938" t="inlineStr"/>
+      <c r="L1938" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Marcar atividade 3862 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -89817,13 +89817,17 @@
         <v>45</v>
       </c>
       <c r="I1938" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="J1938" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K1938" t="inlineStr"/>
-      <c r="L1938" t="inlineStr"/>
+      <c r="L1938" t="inlineStr">
+        <is>
+          <t>2026-09-18 18:21</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Marcar atividade 510 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2567,13 +2567,17 @@
         <v>20</v>
       </c>
       <c r="I43" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>2026-09-19 17:18</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">

</xml_diff>

<commit_message>
Marcar atividade 525 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -3235,13 +3235,17 @@
         <v>30</v>
       </c>
       <c r="I57" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J57" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>2026-09-19 17:19</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">

</xml_diff>

<commit_message>
Marcar atividade 516 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2867,13 +2867,17 @@
         <v>30</v>
       </c>
       <c r="I49" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J49" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>2026-09-21 11:34</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">

</xml_diff>

<commit_message>
Marcar atividade 517 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2917,13 +2917,17 @@
         <v>20</v>
       </c>
       <c r="I50" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J50" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>2026-09-22 10:20</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">

</xml_diff>

<commit_message>
Marcar atividade 518 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2967,13 +2967,17 @@
         <v>20</v>
       </c>
       <c r="I51" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J51" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>2026-09-23 19:35</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">

</xml_diff>

<commit_message>
Marcar atividade 519 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -3017,13 +3017,17 @@
         <v>20</v>
       </c>
       <c r="I52" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J52" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>2026-09-23 19:55</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">

</xml_diff>

<commit_message>
Marcar atividade 520 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -3067,13 +3067,17 @@
         <v>45</v>
       </c>
       <c r="I53" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="J53" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>2026-09-24 02:38</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">

</xml_diff>

<commit_message>
Marcar atividade 521 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -3117,13 +3117,17 @@
         <v>30</v>
       </c>
       <c r="I54" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J54" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>2026-09-25 12:19</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">

</xml_diff>

<commit_message>
Marcar atividade 524 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -3213,13 +3213,17 @@
         <v>20</v>
       </c>
       <c r="I56" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J56" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-09-25 12:19</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">

</xml_diff>

<commit_message>
Marcar atividade 526 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -3313,13 +3313,17 @@
         <v>20</v>
       </c>
       <c r="I58" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J58" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>2026-09-26 02:45</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">

</xml_diff>

<commit_message>
Marcar atividade 522 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -3167,13 +3167,17 @@
         <v>20</v>
       </c>
       <c r="I55" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J55" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-09-29 18:36</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">

</xml_diff>

<commit_message>
Marcar atividade 529 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -3459,13 +3459,17 @@
         <v>20</v>
       </c>
       <c r="I61" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J61" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-09-29 18:36</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">

</xml_diff>

<commit_message>
Marcar atividade 545 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -4199,13 +4199,17 @@
         <v>30</v>
       </c>
       <c r="I77" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J77" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K77" t="inlineStr"/>
-      <c r="L77" t="inlineStr"/>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>2026-09-29 18:36</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">

</xml_diff>

<commit_message>
Marcar atividade 3864 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -63975,13 +63975,17 @@
         <v>30</v>
       </c>
       <c r="I1375" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J1375" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K1375" t="inlineStr"/>
-      <c r="L1375" t="inlineStr"/>
+      <c r="L1375" t="inlineStr">
+        <is>
+          <t>2026-09-30 00:30</t>
+        </is>
+      </c>
     </row>
     <row r="1376">
       <c r="A1376" t="n">

</xml_diff>

<commit_message>
Marcar atividade 3863 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -63929,13 +63929,17 @@
         <v>40</v>
       </c>
       <c r="I1374" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J1374" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K1374" t="inlineStr"/>
-      <c r="L1374" t="inlineStr"/>
+      <c r="L1374" t="inlineStr">
+        <is>
+          <t>2026-09-30 10:34</t>
+        </is>
+      </c>
     </row>
     <row r="1375">
       <c r="A1375" t="n">

</xml_diff>

<commit_message>
Marcar atividade 3865 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -64029,13 +64029,17 @@
         <v>30</v>
       </c>
       <c r="I1376" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J1376" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K1376" t="inlineStr"/>
-      <c r="L1376" t="inlineStr"/>
+      <c r="L1376" t="inlineStr">
+        <is>
+          <t>2026-09-30 11:09</t>
+        </is>
+      </c>
     </row>
     <row r="1377">
       <c r="A1377" t="n">

</xml_diff>

<commit_message>
Adicionar atividade: Duolingo - Tarefas de Hoje  (Darlei Delfino)
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1871"/>
+  <dimension ref="A1:L1872"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -86810,6 +86810,52 @@
       </c>
       <c r="K1871" t="inlineStr"/>
       <c r="L1871" t="inlineStr"/>
+    </row>
+    <row r="1872">
+      <c r="A1872" t="n">
+        <v>4361</v>
+      </c>
+      <c r="B1872" t="inlineStr">
+        <is>
+          <t>Darlei Delfino</t>
+        </is>
+      </c>
+      <c r="C1872" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="D1872" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="E1872" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Duolingo - Tarefas de Hoje </t>
+        </is>
+      </c>
+      <c r="F1872" t="inlineStr">
+        <is>
+          <t>Speaking</t>
+        </is>
+      </c>
+      <c r="G1872" t="inlineStr">
+        <is>
+          <t>Personalizado</t>
+        </is>
+      </c>
+      <c r="H1872" t="n">
+        <v>15</v>
+      </c>
+      <c r="I1872" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1872" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1872" t="inlineStr"/>
+      <c r="L1872" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>